<commit_message>
build(model): regenerate excel financial model with burn-in balance and updated TWCF bridge
</commit_message>
<xml_diff>
--- a/Institutional_Payment_Float_Financial_Model.xlsx
+++ b/Institutional_Payment_Float_Financial_Model.xlsx
@@ -26036,7 +26036,7 @@
         <v>-15604152.4</v>
       </c>
       <c r="F2" s="25" t="n">
-        <v>0</v>
+        <v>19213.41</v>
       </c>
       <c r="G2" s="25" t="n">
         <v>0</v>
@@ -26045,7 +26045,7 @@
         <v>-655544.73</v>
       </c>
       <c r="I2" s="25" t="n">
-        <v>-592758145.4299999</v>
+        <v>-592777358.84</v>
       </c>
       <c r="J2" s="33">
         <f>SUM(E2:I2)</f>
@@ -26076,7 +26076,7 @@
         <v>4517150.09</v>
       </c>
       <c r="F3" s="27" t="n">
-        <v>0</v>
+        <v>-1117481.57</v>
       </c>
       <c r="G3" s="27" t="n">
         <v>0</v>
@@ -26085,7 +26085,7 @@
         <v>-4704991.630000001</v>
       </c>
       <c r="I3" s="27" t="n">
-        <v>89326403.77</v>
+        <v>90443885.34</v>
       </c>
       <c r="J3" s="35">
         <f>SUM(E3:I3)</f>
@@ -26116,7 +26116,7 @@
         <v>5124088.78</v>
       </c>
       <c r="F4" s="25" t="n">
-        <v>0</v>
+        <v>-56221.49</v>
       </c>
       <c r="G4" s="25" t="n">
         <v>0</v>
@@ -26125,7 +26125,7 @@
         <v>-4772843.909999999</v>
       </c>
       <c r="I4" s="25" t="n">
-        <v>219355321.49</v>
+        <v>219411542.98</v>
       </c>
       <c r="J4" s="33">
         <f>SUM(E4:I4)</f>
@@ -26156,7 +26156,7 @@
         <v>4727804.55</v>
       </c>
       <c r="F5" s="27" t="n">
-        <v>0</v>
+        <v>18997.54</v>
       </c>
       <c r="G5" s="27" t="n">
         <v>0</v>
@@ -26165,7 +26165,7 @@
         <v>-4728541.59</v>
       </c>
       <c r="I5" s="27" t="n">
-        <v>226082826.48</v>
+        <v>226063828.93</v>
       </c>
       <c r="J5" s="35">
         <f>SUM(E5:I5)</f>
@@ -26196,7 +26196,7 @@
         <v>5004562.52</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>0</v>
+        <v>-76840.39999999999</v>
       </c>
       <c r="G6" s="25" t="n">
         <v>0</v>
@@ -26205,7 +26205,7 @@
         <v>-4759481.560000002</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>216621708.43</v>
+        <v>216698548.83</v>
       </c>
       <c r="J6" s="33">
         <f>SUM(E6:I6)</f>
@@ -26236,7 +26236,7 @@
         <v>5274686.48</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>0</v>
+        <v>-44866</v>
       </c>
       <c r="G7" s="27" t="n">
         <v>0</v>
@@ -26245,7 +26245,7 @@
         <v>-4789679.869999997</v>
       </c>
       <c r="I7" s="27" t="n">
-        <v>221626221.19</v>
+        <v>221671087.19</v>
       </c>
       <c r="J7" s="35">
         <f>SUM(E7:I7)</f>
@@ -26276,7 +26276,7 @@
         <v>4783200.06</v>
       </c>
       <c r="F8" s="25" t="n">
-        <v>0</v>
+        <v>164107.67</v>
       </c>
       <c r="G8" s="25" t="n">
         <v>0</v>
@@ -26285,7 +26285,7 @@
         <v>-4734734.5</v>
       </c>
       <c r="I8" s="25" t="n">
-        <v>241888100.85</v>
+        <v>241723993.17</v>
       </c>
       <c r="J8" s="33">
         <f>SUM(E8:I8)</f>
@@ -26316,7 +26316,7 @@
         <v>5210224.4</v>
       </c>
       <c r="F9" s="27" t="n">
-        <v>0</v>
+        <v>-84215.99000000001</v>
       </c>
       <c r="G9" s="27" t="n">
         <v>0</v>
@@ -26325,7 +26325,7 @@
         <v>-4782473.390000001</v>
       </c>
       <c r="I9" s="27" t="n">
-        <v>216997110.31</v>
+        <v>217081326.3</v>
       </c>
       <c r="J9" s="35">
         <f>SUM(E9:I9)</f>
@@ -26356,7 +26356,7 @@
         <v>4546105.54</v>
       </c>
       <c r="F10" s="25" t="n">
-        <v>0</v>
+        <v>-3808.37</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>0</v>
@@ -26365,7 +26365,7 @@
         <v>-4708228.670000002</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>222683859.76</v>
+        <v>222687668.13</v>
       </c>
       <c r="J10" s="33">
         <f>SUM(E10:I10)</f>
@@ -26396,7 +26396,7 @@
         <v>4859458.02</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>0</v>
+        <v>-61723.03</v>
       </c>
       <c r="G11" s="27" t="n">
         <v>0</v>
@@ -26405,7 +26405,7 @@
         <v>-4743259.699999996</v>
       </c>
       <c r="I11" s="27" t="n">
-        <v>217418834.91</v>
+        <v>217480557.94</v>
       </c>
       <c r="J11" s="35">
         <f>SUM(E11:I11)</f>
@@ -26436,7 +26436,7 @@
         <v>4870968.5</v>
       </c>
       <c r="F12" s="25" t="n">
-        <v>0</v>
+        <v>331209.47</v>
       </c>
       <c r="G12" s="25" t="n">
         <v>0</v>
@@ -26445,7 +26445,7 @@
         <v>-4744546.510000005</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>260800760.64</v>
+        <v>260469551.17</v>
       </c>
       <c r="J12" s="33">
         <f>SUM(E12:I12)</f>
@@ -26476,7 +26476,7 @@
         <v>4641282.42</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>0</v>
+        <v>-261506.78</v>
       </c>
       <c r="G13" s="27" t="n">
         <v>0</v>
@@ -26485,7 +26485,7 @@
         <v>-4718868.909999996</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>194674711.85</v>
+        <v>194936218.64</v>
       </c>
       <c r="J13" s="35">
         <f>SUM(E13:I13)</f>
@@ -26516,7 +26516,7 @@
         <v>4636083.22</v>
       </c>
       <c r="F14" s="25" t="n">
-        <v>0</v>
+        <v>148045.96</v>
       </c>
       <c r="G14" s="25" t="n">
         <v>0</v>
@@ -26525,7 +26525,7 @@
         <v>-4718287.670000002</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>239344542.17</v>
+        <v>239196496.22</v>
       </c>
       <c r="J14" s="33">
         <f>SUM(E14:I14)</f>
@@ -26556,7 +26556,7 @@
         <v>4954764.85</v>
       </c>
       <c r="F15" s="27" t="n">
-        <v>0</v>
+        <v>-85560.94</v>
       </c>
       <c r="G15" s="27" t="n">
         <v>0</v>
@@ -26565,7 +26565,7 @@
         <v>-4753914.460000001</v>
       </c>
       <c r="I15" s="27" t="n">
-        <v>215246270.46</v>
+        <v>215331831.4</v>
       </c>
       <c r="J15" s="35">
         <f>SUM(E15:I15)</f>
@@ -26596,7 +26596,7 @@
         <v>3769280.73</v>
       </c>
       <c r="F16" s="25" t="n">
-        <v>0</v>
+        <v>36896.83</v>
       </c>
       <c r="G16" s="25" t="n">
         <v>0</v>
@@ -26605,7 +26605,7 @@
         <v>-4621384.109999999</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>223226407.09</v>
+        <v>223189510.26</v>
       </c>
       <c r="J16" s="33">
         <f>SUM(E16:I16)</f>
@@ -26636,7 +26636,7 @@
         <v>4740922.44</v>
       </c>
       <c r="F17" s="27" t="n">
-        <v>0</v>
+        <v>63519.79</v>
       </c>
       <c r="G17" s="27" t="n">
         <v>0</v>
@@ -26645,7 +26645,7 @@
         <v>-4730008.100000001</v>
       </c>
       <c r="I17" s="27" t="n">
-        <v>230664863.07</v>
+        <v>230601343.28</v>
       </c>
       <c r="J17" s="35">
         <f>SUM(E17:I17)</f>
@@ -26676,7 +26676,7 @@
         <v>4457069.12</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>0</v>
+        <v>35429.07</v>
       </c>
       <c r="G18" s="25" t="n">
         <v>0</v>
@@ -26685,7 +26685,7 @@
         <v>-4698274.909999996</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>225751018.48</v>
+        <v>225715589.42</v>
       </c>
       <c r="J18" s="33">
         <f>SUM(E18:I18)</f>
@@ -26716,7 +26716,7 @@
         <v>4702675.26</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>0</v>
+        <v>-111065.46</v>
       </c>
       <c r="G19" s="27" t="n">
         <v>0</v>
@@ -26725,7 +26725,7 @@
         <v>-4725732.280000001</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>210949982.63</v>
+        <v>211061048.09</v>
       </c>
       <c r="J19" s="35">
         <f>SUM(E19:I19)</f>
@@ -26756,7 +26756,7 @@
         <v>5243099.39</v>
       </c>
       <c r="F20" s="25" t="n">
-        <v>0</v>
+        <v>-123301.39</v>
       </c>
       <c r="G20" s="25" t="n">
         <v>0</v>
@@ -26765,7 +26765,7 @@
         <v>-4786148.620000005</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>213383006.71</v>
+        <v>213506308.1</v>
       </c>
       <c r="J20" s="33">
         <f>SUM(E20:I20)</f>
@@ -26796,7 +26796,7 @@
         <v>4106469.52</v>
       </c>
       <c r="F21" s="27" t="n">
-        <v>0</v>
+        <v>184422.41</v>
       </c>
       <c r="G21" s="27" t="n">
         <v>0</v>
@@ -26805,7 +26805,7 @@
         <v>-4659079.86999999</v>
       </c>
       <c r="I21" s="27" t="n">
-        <v>240442453.26</v>
+        <v>240258030.85</v>
       </c>
       <c r="J21" s="35">
         <f>SUM(E21:I21)</f>
@@ -26836,7 +26836,7 @@
         <v>5367225.72</v>
       </c>
       <c r="F22" s="25" t="n">
-        <v>0</v>
+        <v>-174619.13</v>
       </c>
       <c r="G22" s="25" t="n">
         <v>0</v>
@@ -26845,7 +26845,7 @@
         <v>-4800025.230000004</v>
       </c>
       <c r="I22" s="25" t="n">
-        <v>207219010.78</v>
+        <v>207393629.92</v>
       </c>
       <c r="J22" s="33">
         <f>SUM(E22:I22)</f>
@@ -26876,7 +26876,7 @@
         <v>9454169.699999999</v>
       </c>
       <c r="F23" s="27" t="n">
-        <v>0</v>
+        <v>33002.11</v>
       </c>
       <c r="G23" s="27" t="n">
         <v>0</v>
@@ -26885,7 +26885,7 @@
         <v>-4656922.269999996</v>
       </c>
       <c r="I23" s="27" t="n">
-        <v>224969114.26</v>
+        <v>224936112.15</v>
       </c>
       <c r="J23" s="35">
         <f>SUM(E23:I23)</f>

</xml_diff>